<commit_message>
Phase 4 Complete: Formatted manual testing matrix in TestingEvidence document (05-08-2026)
</commit_message>
<xml_diff>
--- a/VolunteerConnect/Docs/VolunteerConnect_IssueTrackingLog.xlsx
+++ b/VolunteerConnect/Docs/VolunteerConnect_IssueTrackingLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\VolunteerConnect\VolunteerConnect\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E126DE1-D28F-4851-B72E-106695118AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACD7E6B-1BED-401C-B746-C3066DD4279E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8964" yWindow="588" windowWidth="13620" windowHeight="11592" xr2:uid="{10BAA2FA-F616-4930-9B9B-F593A5F20FE0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="106">
   <si>
     <t>ISSUE ID:</t>
   </si>
@@ -165,13 +165,783 @@
   </si>
   <si>
     <t>Whitespace inputs correctly blocked.</t>
+  </si>
+  <si>
+    <t>ISS-004</t>
+  </si>
+  <si>
+    <t>Navigation route missing error when tapping opportunity card.</t>
+  </si>
+  <si>
+    <t>Registered routes in AppShell.xaml.cs using Routing.RegisterRoute</t>
+  </si>
+  <si>
+    <t>ISS-005</t>
+  </si>
+  <si>
+    <t>MAUI Compilation</t>
+  </si>
+  <si>
+    <t>Build failed with missing type errors for OpportunityDetailsPage, RegistrationPage, MyRegistrationsPage, EditRegistrationPage, and PrivacyPage.</t>
+  </si>
+  <si>
+    <t>App compiles cleanly after adding page references to MauiProgram.cs and AppShell.cs.</t>
+  </si>
+  <si>
+    <t>Compiler threw CS0246 errors for missing classes in VolunteerConnect.Views.</t>
+  </si>
+  <si>
+    <t>Visual Studio Error List Window</t>
+  </si>
+  <si>
+    <t>AppShell.xaml.cs and MauiProgram.cs declared routing and DI registrations before the XAML ContentPages were added to the project.</t>
+  </si>
+  <si>
+    <t>Created all 5 remaining ContentPage XAML and C# code-behind files in Views/ folder.</t>
+  </si>
+  <si>
+    <t>Project compiles with 0 errors.</t>
+  </si>
+  <si>
+    <t>ISS-006</t>
+  </si>
+  <si>
+    <t>Services / Regex</t>
+  </si>
+  <si>
+    <t>Compiler error on Regex.IsMatch() inside PrivacyValidator.cs.</t>
+  </si>
+  <si>
+    <t>Contact detail validation checks string format without compiler error.</t>
+  </si>
+  <si>
+    <t>Compiler threw error CS0029 regarding non-static/instance invocation of Regex.IsMatch.</t>
+  </si>
+  <si>
+    <t>Visual Studio Compiler / Error List</t>
+  </si>
+  <si>
+    <t>Incorrect overload syntax used when calling Regex.IsMatch() static method.</t>
+  </si>
+  <si>
+    <t>Updated PrivacyValidator.cs to pass pattern string directly into static Regex.IsMatch(input, pattern, options).</t>
+  </si>
+  <si>
+    <t>Valid email and phone inputs return true; invalid inputs return false.</t>
+  </si>
+  <si>
+    <t>SS-007</t>
+  </si>
+  <si>
+    <t>XAML Parsing</t>
+  </si>
+  <si>
+    <t>Build failed on line 17 due to duplicate root tag; C# code-behind lost reference to controls.</t>
+  </si>
+  <si>
+    <t>VS Error List / Output Window</t>
+  </si>
+  <si>
+    <t>Removed duplicate XML root block; executed Clean &amp; Rebuild.</t>
+  </si>
+  <si>
+    <t>Build succeeded with 0 errors; controls properly bound.</t>
+  </si>
+  <si>
+    <t>ISS-008</t>
+  </si>
+  <si>
+    <t>MAUI Build / Compiler</t>
+  </si>
+  <si>
+    <t>Compiler threw multiple CS0229 duplicate symbol errors during build.</t>
+  </si>
+  <si>
+    <t>VS Error List / File Explorer Audit</t>
+  </si>
+  <si>
+    <t>Build succeeded with 0 errors; ambiguous symbol warnings cleared.</t>
+  </si>
+  <si>
+    <t>ISS-009</t>
+  </si>
+  <si>
+    <t>Visual Studio IDE</t>
+  </si>
+  <si>
+    <t>"There were build errors" execution dialog prompt appeared when hitting F5.</t>
+  </si>
+  <si>
+    <t>App builds with zero errors and launches updated assembly on emulator.</t>
+  </si>
+  <si>
+    <t>IDE prompted to run last successful build due to unhandled compiler errors in active build configuration.</t>
+  </si>
+  <si>
+    <t>VS Error List Audit / Output Window</t>
+  </si>
+  <si>
+    <t>Solution attempted deployment while stashed build artifacts or missing view registrations remained unresolved in active configuration.</t>
+  </si>
+  <si>
+    <t>Cancelled execution, reviewed Error List, closed open XAML tabs, and performed full Rebuild Solution.</t>
+  </si>
+  <si>
+    <t>Project built cleanly with zero errors; application launched on target emulator.</t>
+  </si>
+  <si>
+    <t>ISS-010</t>
+  </si>
+  <si>
+    <t>MSBuild / MAUI Imports</t>
+  </si>
+  <si>
+    <t>Clean build and deployment to emulator without process lock exceptions.</t>
+  </si>
+  <si>
+    <t>Task Manager Audit / VS Error List</t>
+  </si>
+  <si>
+    <t>Solution built cleanly with 0 errors; app deployed successfully.</t>
+  </si>
+  <si>
+    <t>ISS-011</t>
+  </si>
+  <si>
+    <t>Compiler generated duplicate symbol definitions in intermediate build files prior to Rebuild execution.</t>
+  </si>
+  <si>
+    <t>Intermediate build artifacts lingering during active Clean/Rebuild cycle before full compiler cache refresh.</t>
+  </si>
+  <si>
+    <t>Project compiled cleanly with 0 errors; application running on target emulator.</t>
+  </si>
+  <si>
+    <r>
+      <t>OpportunityDetailsPage.xaml</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> threw unexpected XML declaration parser error and missing control name errors.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>XAML parses cleanly and binds named labels (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TitleLabel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DateLabel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, etc.) to code-behind.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Duplicate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;?xml ...?&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> declaration and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;ContentPage&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> root tag accidentally pasted into </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage.xaml</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CS0229 ambiguous reference errors between </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage.InitializeComponent()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and controls (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>TitleLabel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>DateLabel</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, etc.).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Clean compilation with a single auto-generated partial class for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Stale auto-generated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.g.cs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> files remained in local </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obj</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> directory after resolving XAML syntax error, causing duplicate symbol declarations.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Closed Visual Studio, purged local </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>bin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obj</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> build directories, reopened solution, and executed full Rebuild.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">MSBuild file lock errors on Windows MsixContent DLLs and missing namespace errors for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>QueryProperty</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ContentPage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Build failed with file access lock exceptions in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obj\Debug\</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and CS0246 missing namespace errors in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage.xaml.cs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Background </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MSBuild.exe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> processes locked intermediate </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obj</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> output files; missing </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Microsoft.Maui.Controls</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> namespace import in code-behind.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Terminated MSBuild tasks, deleted </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>bin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>obj</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> directories, added </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>using Microsoft.Maui.Controls;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage.xaml.cs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, and executed Rebuild.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">CS0229 ambiguous symbol errors between </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage.InitializeComponent()</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and control fields after Solution Clean.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Solution compiles with single auto-generated partial class file for </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>OpportunityDetailsPage</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Executed full Rebuild Solution to regenerate unified </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.g.cs</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> partial classes across all 7 Views.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,6 +957,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -196,7 +980,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -204,29 +988,53 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFC4C7C5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -234,39 +1042,17 @@
   </cellStyles>
   <dxfs count="14">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -289,6 +1075,171 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -305,21 +1256,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CAF8E8DF-50C0-4A74-8A5A-EF21BDFB1D0C}" name="Table1" displayName="Table1" ref="B7:M32" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CAF8E8DF-50C0-4A74-8A5A-EF21BDFB1D0C}" name="Table1" displayName="Table1" ref="B7:M32" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
   <autoFilter ref="B7:M32" xr:uid="{CAF8E8DF-50C0-4A74-8A5A-EF21BDFB1D0C}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{136170E2-DD45-4A5E-85FE-634DEE69C417}" name="ISSUE ID:" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{6879624A-0FDF-4F1A-A689-16D636C24372}" name="DATE IDENTIFIED:" dataDxfId="10"/>
-    <tableColumn id="3" xr3:uid="{9AB7AAE1-EC47-42EF-8414-FA4728F77ACE}" name="FEATURE:" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{7FAE14F0-B231-467B-B6D8-3C91BE855798}" name="DESCRIPTION:" dataDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{8ACD74F5-44AA-4092-BDCA-7BF22DEE67A0}" name="EXPECTED RESULT:" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{9453CA77-FA5F-4B42-8F9A-E86EBCB7C1F4}" name="ACTUAL RESULT:" dataDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{826AB988-C84C-4D6E-AAC8-91E18692B8DA}" name="PRIORITY:" dataDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{367DA86B-7F78-4EA5-8D4B-2002C0E449F8}" name="DEBUGGING METHOD:" dataDxfId="4"/>
-    <tableColumn id="9" xr3:uid="{87DCBE5D-3609-4E56-8981-E557FA3E6110}" name="CAUSE:" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{8FC441DA-1064-4460-A5A3-056FE237A0F4}" name="FIX APPLIED:" dataDxfId="2"/>
-    <tableColumn id="11" xr3:uid="{B041CFA9-8DB6-4EEB-A597-470B4DCBC1A8}" name="RETEST RESULT:" dataDxfId="0"/>
-    <tableColumn id="12" xr3:uid="{C786C6BE-9718-4861-9E32-10EB4B57B368}" name="STATUS:" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{6879624A-0FDF-4F1A-A689-16D636C24372}" name="DATE IDENTIFIED:" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{9AB7AAE1-EC47-42EF-8414-FA4728F77ACE}" name="FEATURE:" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{7FAE14F0-B231-467B-B6D8-3C91BE855798}" name="DESCRIPTION:" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{8ACD74F5-44AA-4092-BDCA-7BF22DEE67A0}" name="EXPECTED RESULT:" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{9453CA77-FA5F-4B42-8F9A-E86EBCB7C1F4}" name="ACTUAL RESULT:" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{826AB988-C84C-4D6E-AAC8-91E18692B8DA}" name="PRIORITY:" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{367DA86B-7F78-4EA5-8D4B-2002C0E449F8}" name="DEBUGGING METHOD:" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{87DCBE5D-3609-4E56-8981-E557FA3E6110}" name="CAUSE:" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{8FC441DA-1064-4460-A5A3-056FE237A0F4}" name="FIX APPLIED:" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{B041CFA9-8DB6-4EEB-A597-470B4DCBC1A8}" name="RETEST RESULT:" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{C786C6BE-9718-4861-9E32-10EB4B57B368}" name="STATUS:" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -642,14 +1593,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A6FB081-C45D-4506-885B-05BF409D2650}">
-  <dimension ref="B7:M10"/>
+  <dimension ref="B7:M21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="3"/>
     <col min="2" max="2" width="12.5546875" style="3" customWidth="1"/>
     <col min="3" max="3" width="21.5546875" style="3" customWidth="1"/>
     <col min="4" max="4" width="15.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.5546875" style="6" customWidth="1"/>
+    <col min="5" max="5" width="24" style="6" customWidth="1"/>
     <col min="6" max="6" width="23.21875" style="6" customWidth="1"/>
     <col min="7" max="7" width="22.44140625" style="6" customWidth="1"/>
     <col min="8" max="8" width="22.44140625" style="3" customWidth="1"/>
@@ -661,41 +1612,41 @@
     <col min="14" max="16384" width="8.88671875" style="3"/>
   </cols>
   <sheetData>
-    <row r="7" spans="2:13" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.3">
-      <c r="B7" s="2" t="s">
+    <row r="7" spans="2:13" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="1" t="s">
         <v>11</v>
       </c>
     </row>
@@ -706,7 +1657,7 @@
       <c r="C8" s="4">
         <v>46239</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="5" t="s">
         <v>13</v>
       </c>
       <c r="E8" s="6" t="s">
@@ -813,6 +1764,292 @@
         <v>22</v>
       </c>
     </row>
+    <row r="11" spans="2:13" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="4">
+        <v>46239</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="2:13" ht="102.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="4">
+        <v>46239</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="K12" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="2:13" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="4">
+        <v>46239</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="L13" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="2:13" ht="99.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C14" s="8">
+        <v>46239</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="H14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="K14" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="M14" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="2:13" ht="100.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="8">
+        <v>46239</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" ht="83.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="8">
+        <v>46239</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="K16" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="M16" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" ht="103.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="8">
+        <v>46239</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K17" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="M17" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" ht="85.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="8">
+        <v>46239</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H18" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" ht="102" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="20" spans="2:13" ht="86.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="21" spans="2:13" ht="85.8" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Phase 5 Complete: Integrated xUnit test project VolunteerConnect.Tests, updated issue log (ISS-001 to ISS-013) and testing evidence (07-08-2026)
</commit_message>
<xml_diff>
--- a/VolunteerConnect/Docs/VolunteerConnect_IssueTrackingLog.xlsx
+++ b/VolunteerConnect/Docs/VolunteerConnect_IssueTrackingLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\VolunteerConnect\VolunteerConnect\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ACD7E6B-1BED-401C-B746-C3066DD4279E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A188B00C-F188-4047-9A98-32E3949F879D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8964" yWindow="588" windowWidth="13620" windowHeight="11592" xr2:uid="{10BAA2FA-F616-4930-9B9B-F593A5F20FE0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="123">
   <si>
     <t>ISSUE ID:</t>
   </si>
@@ -935,6 +935,57 @@
       </rPr>
       <t xml:space="preserve"> partial classes across all 7 Views.</t>
     </r>
+  </si>
+  <si>
+    <t>ISS-012</t>
+  </si>
+  <si>
+    <t>Unit Testing</t>
+  </si>
+  <si>
+    <t>"There were build errors" dialog prompt appeared when attempting to execute xUnit tests.</t>
+  </si>
+  <si>
+    <t>Test assembly compiles and executes xUnit tests for PrivacyValidator.</t>
+  </si>
+  <si>
+    <t>Test project failed to compile due to missing accessibility modifier on validation class.</t>
+  </si>
+  <si>
+    <t>VS Error List / Test Explorer Audit</t>
+  </si>
+  <si>
+    <t>PrivacyValidator utility class lacked public modifier, preventing VolunteerConnect.Tests assembly from referencing validation methods.</t>
+  </si>
+  <si>
+    <t>Added public modifier to PrivacyValidator.cs and updated parameters to accept nullable strings (string?).</t>
+  </si>
+  <si>
+    <t>All unit tests passed successfully with 0 compiler errors.</t>
+  </si>
+  <si>
+    <t>ISS-013</t>
+  </si>
+  <si>
+    <t>Unit Testing / MAUI</t>
+  </si>
+  <si>
+    <t>CS0229 ambiguous symbol errors and project incompatibility error (.NETCoreApp v9.0 vs multi-targeted MAUI).</t>
+  </si>
+  <si>
+    <t>Test project compiles and runs unit tests for validation rules smoothly.</t>
+  </si>
+  <si>
+    <t>MSBuild generated duplicate .g.cs partial classes and threw framework mismatch errors when referencing MAUI app project directly.</t>
+  </si>
+  <si>
+    <t>Referencing a multi-targeted MAUI UI project directly inside a standard xUnit runner caused XAML code generator collisions across platform builds.</t>
+  </si>
+  <si>
+    <t>Configured VolunteerConnect.Tests.csproj to compile PrivacyValidator.cs directly as a linked file, isolating validation logic from XAML builds.</t>
+  </si>
+  <si>
+    <t>All 16 unit tests passed in Test Explorer in 403 ms with 0 build errors.</t>
   </si>
 </sst>
 </file>
@@ -1007,34 +1058,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1053,7 +1095,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1072,21 +1114,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1156,7 +1184,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1212,7 +1240,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1226,7 +1254,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1240,7 +1268,21 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1596,20 +1638,19 @@
   <dimension ref="B7:M21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="3"/>
-    <col min="2" max="2" width="12.5546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="15.5546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24" style="6" customWidth="1"/>
-    <col min="6" max="6" width="23.21875" style="6" customWidth="1"/>
-    <col min="7" max="7" width="22.44140625" style="6" customWidth="1"/>
-    <col min="8" max="8" width="22.44140625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="26.6640625" style="6" customWidth="1"/>
-    <col min="10" max="10" width="25.6640625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="26" style="6" customWidth="1"/>
-    <col min="12" max="12" width="19.6640625" style="6" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" style="3" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="3"/>
+    <col min="1" max="1" width="8.88671875" style="2"/>
+    <col min="2" max="2" width="12.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="15.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24" style="2" customWidth="1"/>
+    <col min="6" max="6" width="23.21875" style="2" customWidth="1"/>
+    <col min="7" max="8" width="22.44140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="25.6640625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="26" style="2" customWidth="1"/>
+    <col min="12" max="12" width="19.6640625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="11.44140625" style="2" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
     <row r="7" spans="2:13" s="1" customFormat="1" ht="18" x14ac:dyDescent="0.3">
@@ -1622,28 +1663,28 @@
       <c r="D7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="1" t="s">
         <v>10</v>
       </c>
       <c r="M7" s="1" t="s">
@@ -1651,404 +1692,478 @@
       </c>
     </row>
     <row r="8" spans="2:13" ht="114" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8" s="6">
         <v>46239</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="I8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="6" t="s">
+      <c r="J8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="K8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="L8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="M8" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="9" spans="2:13" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="6">
         <v>46239</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="H9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="I9" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="L9" s="6" t="s">
+      <c r="L9" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="M9" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="2:13" ht="102" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C10" s="6">
         <v>46239</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="H10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="6" t="s">
+      <c r="I10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="J10" s="6" t="s">
+      <c r="J10" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="K10" s="6" t="s">
+      <c r="K10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="L10" s="6" t="s">
+      <c r="L10" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="M10" s="3" t="s">
+      <c r="M10" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="2:13" ht="88.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="6">
         <v>46239</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="I11" s="6" t="s">
+      <c r="I11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="M11" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="12" spans="2:13" ht="102.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12" s="6">
         <v>46239</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="H12" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="6" t="s">
+      <c r="I12" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="J12" s="6" t="s">
+      <c r="J12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="K12" s="6" t="s">
+      <c r="K12" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L12" s="6" t="s">
+      <c r="L12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="M12" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" spans="2:13" ht="102" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13" s="6">
         <v>46239</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="H13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="J13" s="6" t="s">
+      <c r="J13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="K13" s="6" t="s">
+      <c r="K13" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="L13" s="6" t="s">
+      <c r="L13" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="M13" s="3" t="s">
+      <c r="M13" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" spans="2:13" ht="99.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="4">
         <v>46239</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="J14" s="7" t="s">
+      <c r="J14" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="K14" s="7" t="s">
+      <c r="K14" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="L14" s="7" t="s">
+      <c r="L14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="M14" s="7" t="s">
+      <c r="M14" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="2:13" ht="100.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="4">
         <v>46239</v>
       </c>
-      <c r="D15" s="7" t="s">
+      <c r="D15" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="E15" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="H15" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="J15" s="7" t="s">
+      <c r="J15" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="K15" s="7" t="s">
+      <c r="K15" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="L15" s="7" t="s">
+      <c r="L15" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="M15" s="7" t="s">
+      <c r="M15" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="2:13" ht="83.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="4">
         <v>46239</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="D16" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="E16" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="F16" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="H16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="J16" s="7" t="s">
+      <c r="J16" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="K16" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="L16" s="7" t="s">
+      <c r="L16" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="M16" s="7" t="s">
+      <c r="M16" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="17" spans="2:13" ht="103.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="4">
         <v>46239</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="D17" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="E17" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="G17" s="7" t="s">
+      <c r="G17" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="J17" s="7" t="s">
+      <c r="J17" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="K17" s="7" t="s">
+      <c r="K17" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="L17" s="7" t="s">
+      <c r="L17" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="M17" s="7" t="s">
+      <c r="M17" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="2:13" ht="85.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="4">
         <v>46239</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D18" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="E18" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G18" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="J18" s="7" t="s">
+      <c r="J18" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="K18" s="7" t="s">
+      <c r="K18" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="L18" s="7" t="s">
+      <c r="L18" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="M18" s="7" t="s">
+      <c r="M18" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="2:13" ht="102" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="2:13" ht="86.4" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="19" spans="2:13" ht="102" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" s="6">
+        <v>46241</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C20" s="6">
+        <v>46241</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
     <row r="21" spans="2:13" ht="85.8" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>